<commit_message>
fix(api.main): Added type check suppresion
</commit_message>
<xml_diff>
--- a/data/templates/output_template.xlsx
+++ b/data/templates/output_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnirbanDas\Documents\AniDas\PMI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\anirban\workspace\projects\rpa-complexity-agent\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D343C058-842C-46E9-9A9F-48065CBDFEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2996ABB5-94A7-4317-B622-46B10EB56FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3407,126 +3407,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="46" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3578,17 +3458,137 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="46" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4237,50 +4237,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>2609850</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1792816" cy="1206917"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A9EC0A8-D59B-4EEF-8098-6CD82BD17D9E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9782175" y="1"/>
-          <a:ext cx="1792816" cy="1206917"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -12295,6 +12251,9 @@
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Calculator"/>
       <sheetName val="Feature and delivery timeline"/>
@@ -12737,23 +12696,23 @@
       <c r="D7" s="5"/>
     </row>
     <row r="8" spans="2:26" s="107" customFormat="1" ht="15.75" thickBot="1">
-      <c r="D8" s="227" t="s">
+      <c r="D8" s="187" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="228"/>
-      <c r="F8" s="228"/>
-      <c r="G8" s="228"/>
-      <c r="H8" s="228"/>
-      <c r="I8" s="228"/>
-      <c r="J8" s="228"/>
-      <c r="K8" s="228"/>
-      <c r="L8" s="228"/>
-      <c r="M8" s="228"/>
-      <c r="N8" s="228"/>
-      <c r="O8" s="228"/>
-      <c r="P8" s="228"/>
-      <c r="Q8" s="228"/>
-      <c r="R8" s="229"/>
+      <c r="E8" s="188"/>
+      <c r="F8" s="188"/>
+      <c r="G8" s="188"/>
+      <c r="H8" s="188"/>
+      <c r="I8" s="188"/>
+      <c r="J8" s="188"/>
+      <c r="K8" s="188"/>
+      <c r="L8" s="188"/>
+      <c r="M8" s="188"/>
+      <c r="N8" s="188"/>
+      <c r="O8" s="188"/>
+      <c r="P8" s="188"/>
+      <c r="Q8" s="188"/>
+      <c r="R8" s="189"/>
     </row>
     <row r="9" spans="2:26" s="154" customFormat="1" ht="50.25" thickBot="1">
       <c r="D9" s="161" t="s">
@@ -12866,11 +12825,11 @@
       <c r="V10" s="26">
         <v>8</v>
       </c>
-      <c r="X10" s="213" t="s">
+      <c r="X10" s="222" t="s">
         <v>20</v>
       </c>
-      <c r="Y10" s="213"/>
-      <c r="Z10" s="213"/>
+      <c r="Y10" s="222"/>
+      <c r="Z10" s="222"/>
     </row>
     <row r="11" spans="2:26" s="27" customFormat="1" ht="48">
       <c r="B11" s="22">
@@ -13294,34 +13253,34 @@
       </c>
     </row>
     <row r="25" spans="2:22" s="107" customFormat="1" ht="16.5" thickBot="1">
-      <c r="B25" s="211" t="s">
+      <c r="B25" s="246" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="212"/>
-      <c r="D25" s="230" t="s">
+      <c r="C25" s="247"/>
+      <c r="D25" s="190" t="s">
         <v>114</v>
       </c>
-      <c r="E25" s="231"/>
+      <c r="E25" s="191"/>
       <c r="F25" s="139"/>
-      <c r="G25" s="195" t="s">
+      <c r="G25" s="231" t="s">
         <v>6</v>
       </c>
-      <c r="H25" s="196"/>
+      <c r="H25" s="232"/>
       <c r="I25" s="138"/>
-      <c r="J25" s="193" t="s">
+      <c r="J25" s="229" t="s">
         <v>8</v>
       </c>
-      <c r="K25" s="194"/>
+      <c r="K25" s="230"/>
       <c r="L25" s="138"/>
-      <c r="M25" s="191" t="s">
+      <c r="M25" s="227" t="s">
         <v>9</v>
       </c>
-      <c r="N25" s="192"/>
+      <c r="N25" s="228"/>
       <c r="O25" s="138"/>
-      <c r="P25" s="189" t="s">
+      <c r="P25" s="225" t="s">
         <v>10</v>
       </c>
-      <c r="Q25" s="190"/>
+      <c r="Q25" s="226"/>
       <c r="R25" s="109"/>
       <c r="S25" s="108"/>
       <c r="T25" s="108"/>
@@ -13329,194 +13288,194 @@
       <c r="V25" s="108"/>
     </row>
     <row r="26" spans="2:22">
-      <c r="B26" s="225" t="s">
+      <c r="B26" s="220" t="s">
         <v>113</v>
       </c>
-      <c r="C26" s="226"/>
-      <c r="D26" s="242">
+      <c r="C26" s="221"/>
+      <c r="D26" s="202">
         <v>3</v>
       </c>
-      <c r="E26" s="243"/>
+      <c r="E26" s="203"/>
       <c r="F26" s="137"/>
-      <c r="G26" s="209" t="s">
+      <c r="G26" s="244" t="s">
         <v>112</v>
       </c>
-      <c r="H26" s="210"/>
+      <c r="H26" s="245"/>
       <c r="I26" s="134"/>
-      <c r="J26" s="216">
+      <c r="J26" s="210">
         <v>15</v>
       </c>
-      <c r="K26" s="216"/>
+      <c r="K26" s="210"/>
       <c r="L26" s="134"/>
-      <c r="M26" s="216">
+      <c r="M26" s="210">
         <v>20</v>
       </c>
-      <c r="N26" s="216"/>
+      <c r="N26" s="210"/>
       <c r="O26" s="134"/>
-      <c r="P26" s="216">
+      <c r="P26" s="210">
         <v>25</v>
       </c>
-      <c r="Q26" s="247"/>
+      <c r="Q26" s="211"/>
       <c r="R26" s="1"/>
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="2:22">
-      <c r="B27" s="223" t="s">
+      <c r="B27" s="218" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="224"/>
-      <c r="D27" s="240">
+      <c r="C27" s="219"/>
+      <c r="D27" s="200">
         <v>5</v>
       </c>
-      <c r="E27" s="241"/>
+      <c r="E27" s="201"/>
       <c r="F27" s="136"/>
-      <c r="G27" s="207" t="s">
+      <c r="G27" s="242" t="s">
         <v>110</v>
       </c>
-      <c r="H27" s="208"/>
+      <c r="H27" s="243"/>
       <c r="I27" s="134"/>
-      <c r="J27" s="215">
+      <c r="J27" s="208">
         <v>25</v>
       </c>
-      <c r="K27" s="215"/>
+      <c r="K27" s="208"/>
       <c r="L27" s="134"/>
-      <c r="M27" s="215">
+      <c r="M27" s="208">
         <v>30</v>
       </c>
-      <c r="N27" s="215"/>
+      <c r="N27" s="208"/>
       <c r="O27" s="134"/>
-      <c r="P27" s="215">
+      <c r="P27" s="208">
         <v>40</v>
       </c>
-      <c r="Q27" s="246"/>
+      <c r="Q27" s="209"/>
       <c r="R27" s="1"/>
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="2:22">
-      <c r="B28" s="221" t="s">
+      <c r="B28" s="216" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="222"/>
-      <c r="D28" s="238">
+      <c r="C28" s="217"/>
+      <c r="D28" s="198">
         <v>1</v>
       </c>
-      <c r="E28" s="239"/>
+      <c r="E28" s="199"/>
       <c r="F28" s="135"/>
-      <c r="G28" s="207" t="s">
+      <c r="G28" s="242" t="s">
         <v>108</v>
       </c>
-      <c r="H28" s="208"/>
+      <c r="H28" s="243"/>
       <c r="I28" s="134"/>
-      <c r="J28" s="215">
+      <c r="J28" s="208">
         <v>5</v>
       </c>
-      <c r="K28" s="215"/>
+      <c r="K28" s="208"/>
       <c r="L28" s="134"/>
-      <c r="M28" s="215">
+      <c r="M28" s="208">
         <v>5</v>
       </c>
-      <c r="N28" s="215"/>
+      <c r="N28" s="208"/>
       <c r="O28" s="134"/>
-      <c r="P28" s="215">
+      <c r="P28" s="208">
         <v>10</v>
       </c>
-      <c r="Q28" s="246"/>
+      <c r="Q28" s="209"/>
       <c r="R28" s="1"/>
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="2:22" ht="15.75" thickBot="1">
-      <c r="B29" s="219" t="s">
+      <c r="B29" s="214" t="s">
         <v>107</v>
       </c>
-      <c r="C29" s="220"/>
-      <c r="D29" s="236">
+      <c r="C29" s="215"/>
+      <c r="D29" s="196">
         <v>1</v>
       </c>
-      <c r="E29" s="237"/>
+      <c r="E29" s="197"/>
       <c r="F29" s="133"/>
-      <c r="G29" s="205" t="s">
+      <c r="G29" s="240" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="206"/>
+      <c r="H29" s="241"/>
       <c r="I29" s="132"/>
-      <c r="J29" s="214">
+      <c r="J29" s="205">
         <v>5</v>
       </c>
-      <c r="K29" s="214"/>
+      <c r="K29" s="205"/>
       <c r="L29" s="132"/>
-      <c r="M29" s="214">
+      <c r="M29" s="205">
         <v>5</v>
       </c>
-      <c r="N29" s="214"/>
+      <c r="N29" s="205"/>
       <c r="O29" s="132"/>
-      <c r="P29" s="214">
+      <c r="P29" s="205">
         <v>5</v>
       </c>
-      <c r="Q29" s="245"/>
+      <c r="Q29" s="207"/>
       <c r="R29" s="1"/>
       <c r="S29" s="2"/>
     </row>
     <row r="30" spans="2:22" ht="16.5" thickTop="1" thickBot="1">
-      <c r="B30" s="217" t="s">
+      <c r="B30" s="212" t="s">
         <v>105</v>
       </c>
-      <c r="C30" s="218"/>
-      <c r="D30" s="234">
+      <c r="C30" s="213"/>
+      <c r="D30" s="194">
         <v>10</v>
       </c>
-      <c r="E30" s="235"/>
+      <c r="E30" s="195"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="203" t="s">
+      <c r="G30" s="238" t="s">
         <v>104</v>
       </c>
-      <c r="H30" s="204"/>
+      <c r="H30" s="239"/>
       <c r="I30" s="131"/>
-      <c r="J30" s="202">
+      <c r="J30" s="204">
         <v>50</v>
       </c>
-      <c r="K30" s="202"/>
+      <c r="K30" s="204"/>
       <c r="L30" s="131"/>
-      <c r="M30" s="202">
+      <c r="M30" s="204">
         <v>60</v>
       </c>
-      <c r="N30" s="202"/>
+      <c r="N30" s="204"/>
       <c r="O30" s="131"/>
-      <c r="P30" s="202">
+      <c r="P30" s="204">
         <v>80</v>
       </c>
-      <c r="Q30" s="244"/>
+      <c r="Q30" s="206"/>
       <c r="R30" s="1"/>
       <c r="S30" s="2"/>
     </row>
     <row r="31" spans="2:22" s="125" customFormat="1" ht="30" customHeight="1" thickBot="1">
-      <c r="B31" s="187" t="s">
+      <c r="B31" s="223" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="188"/>
-      <c r="D31" s="232">
+      <c r="C31" s="224"/>
+      <c r="D31" s="192">
         <v>1</v>
       </c>
-      <c r="E31" s="233"/>
+      <c r="E31" s="193"/>
       <c r="F31" s="130"/>
-      <c r="G31" s="200" t="s">
+      <c r="G31" s="236" t="s">
         <v>102</v>
       </c>
-      <c r="H31" s="201"/>
+      <c r="H31" s="237"/>
       <c r="I31" s="129"/>
-      <c r="J31" s="199">
+      <c r="J31" s="235">
         <v>5</v>
       </c>
-      <c r="K31" s="199"/>
+      <c r="K31" s="235"/>
       <c r="L31" s="129"/>
-      <c r="M31" s="199">
+      <c r="M31" s="235">
         <v>6</v>
       </c>
-      <c r="N31" s="199"/>
+      <c r="N31" s="235"/>
       <c r="O31" s="128"/>
-      <c r="P31" s="197">
+      <c r="P31" s="233">
         <v>8</v>
       </c>
-      <c r="Q31" s="198"/>
+      <c r="Q31" s="234"/>
       <c r="R31" s="127"/>
       <c r="S31" s="126"/>
     </row>
@@ -13711,34 +13670,6 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:R8"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="P28:Q28"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="P27:Q27"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="X10:Z10"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="M26:N26"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="P25:Q25"/>
     <mergeCell ref="M25:N25"/>
@@ -13755,6 +13686,34 @@
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="B25:C25"/>
+    <mergeCell ref="X10:Z10"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D8:R8"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="P27:Q27"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E14 K10:K14 Q10:Q14 N10:N14 H10:H14" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -13763,7 +13722,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>